<commit_message>
fix(xlsx, ods, pptx, odp): sixth review fixes for links
- Every link a cell cannot hold is reported, beside the one it does (a bookmark or an address too
  long after a written link went unreported).
- Places are found by an index of the sheets' names: many links over many sheets took time in their
  product.
- A range (#Sheet!A1:C3, ODF's #Sheet.A1:Sheet.C3) is written whole.
- An address's length is measured as it is written (encoded).
- A link relative to the file is written, as DOCX output writes it; a script's is not.
</commit_message>
<xml_diff>
--- a/test/generator/baseline/gen.epub.to.xlsx.xlsx
+++ b/test/generator/baseline/gen.epub.to.xlsx.xlsx
@@ -1227,7 +1227,22 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A30" r:id="rId1"/>
+    <hyperlink ref="A25" r:id="rId1"/>
+    <hyperlink ref="A30" r:id="rId2"/>
+    <hyperlink ref="A33" r:id="rId3"/>
+    <hyperlink ref="A34" r:id="rId4"/>
+    <hyperlink ref="A35" r:id="rId5"/>
+    <hyperlink ref="A36" r:id="rId6"/>
+    <hyperlink ref="A37" r:id="rId7"/>
+    <hyperlink ref="A38" r:id="rId8"/>
+    <hyperlink ref="A44" r:id="rId9"/>
+    <hyperlink ref="A45" r:id="rId10"/>
+    <hyperlink ref="A46" r:id="rId11"/>
+    <hyperlink ref="A47" r:id="rId12"/>
+    <hyperlink ref="A48" r:id="rId13"/>
+    <hyperlink ref="A49" r:id="rId14"/>
+    <hyperlink ref="A82" r:id="rId15"/>
+    <hyperlink ref="A84" r:id="rId16"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>